<commit_message>
Fix XE, Instarem and Remitly collectors from first live run
- XE: skip methods it marks unavailable (bank transfer under €1,000), use
  totalFees, and count the fee inside the amount sent like the manual rows
- Instarem: read the pay-in method name from "text"
- Remitly: blocks GitHub's IPs (429), so fall back to Wise comparison data
- Wise comparison: fall back to all countries, list available aliases on miss
- Remove the 15 XE rows from the first run, which counted the fee wrongly

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018ogxhrLjz2PWd89TeAujLA
</commit_message>
<xml_diff>
--- a/data/EURINR_data.xlsx
+++ b/data/EURINR_data.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O999"/>
+  <dimension ref="A1:O984"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="167.25" customWidth="1" style="23" min="15" max="15"/>
@@ -7177,754 +7177,64 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B147" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C147" s="5" t="inlineStr">
-        <is>
-          <t>bank transfer</t>
-        </is>
-      </c>
-      <c r="D147" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="E147" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F147" s="9" t="n"/>
-      <c r="G147" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H147" s="12" t="n">
-        <v>10821.75</v>
-      </c>
-      <c r="I147" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="J147" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K147" s="10" t="n"/>
-      <c r="L147" s="15">
-        <f>IF(OR(E147="",J147=""),"",(E147-J147)/E147)</f>
-        <v/>
-      </c>
-      <c r="M147" s="15" t="n"/>
-      <c r="N147" s="10" t="n"/>
-      <c r="O147" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: BankTransfer | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L147" s="22" t="n"/>
+      <c r="M147" s="22" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B148" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C148" s="5" t="inlineStr">
-        <is>
-          <t>bank transfer</t>
-        </is>
-      </c>
-      <c r="D148" s="8" t="n">
-        <v>500</v>
-      </c>
-      <c r="E148" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F148" s="9" t="n"/>
-      <c r="G148" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H148" s="12" t="n">
-        <v>54108.75</v>
-      </c>
-      <c r="I148" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="J148" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K148" s="10" t="n"/>
-      <c r="L148" s="15">
-        <f>IF(OR(E148="",J148=""),"",(E148-J148)/E148)</f>
-        <v/>
-      </c>
-      <c r="M148" s="15" t="n"/>
-      <c r="N148" s="10" t="n"/>
-      <c r="O148" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: BankTransfer | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L148" s="22" t="n"/>
+      <c r="M148" s="22" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B149" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C149" s="5" t="inlineStr">
-        <is>
-          <t>bank transfer</t>
-        </is>
-      </c>
-      <c r="D149" s="8" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E149" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F149" s="9" t="n"/>
-      <c r="G149" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H149" s="12" t="n">
-        <v>108217.5</v>
-      </c>
-      <c r="I149" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J149" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K149" s="10" t="n"/>
-      <c r="L149" s="15">
-        <f>IF(OR(E149="",J149=""),"",(E149-J149)/E149)</f>
-        <v/>
-      </c>
-      <c r="M149" s="15" t="n"/>
-      <c r="N149" s="10" t="n"/>
-      <c r="O149" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: BankTransfer | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L149" s="22" t="n"/>
+      <c r="M149" s="22" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B150" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C150" s="5" t="inlineStr">
-        <is>
-          <t>bank transfer</t>
-        </is>
-      </c>
-      <c r="D150" s="8" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E150" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F150" s="9" t="n"/>
-      <c r="G150" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H150" s="12" t="n">
-        <v>216435</v>
-      </c>
-      <c r="I150" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J150" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K150" s="10" t="n"/>
-      <c r="L150" s="15">
-        <f>IF(OR(E150="",J150=""),"",(E150-J150)/E150)</f>
-        <v/>
-      </c>
-      <c r="M150" s="15" t="n"/>
-      <c r="N150" s="10" t="n"/>
-      <c r="O150" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: BankTransfer | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L150" s="22" t="n"/>
+      <c r="M150" s="22" t="n"/>
     </row>
     <row r="151">
-      <c r="A151" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B151" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C151" s="5" t="inlineStr">
-        <is>
-          <t>bank transfer</t>
-        </is>
-      </c>
-      <c r="D151" s="8" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E151" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F151" s="9" t="n"/>
-      <c r="G151" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H151" s="12" t="n">
-        <v>541087.5</v>
-      </c>
-      <c r="I151" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J151" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K151" s="10" t="n"/>
-      <c r="L151" s="15">
-        <f>IF(OR(E151="",J151=""),"",(E151-J151)/E151)</f>
-        <v/>
-      </c>
-      <c r="M151" s="15" t="n"/>
-      <c r="N151" s="10" t="n"/>
-      <c r="O151" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: BankTransfer | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L151" s="22" t="n"/>
+      <c r="M151" s="22" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B152" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C152" s="5" t="inlineStr">
-        <is>
-          <t>debit card</t>
-        </is>
-      </c>
-      <c r="D152" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="E152" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F152" s="9" t="n"/>
-      <c r="G152" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H152" s="12" t="n">
-        <v>10821.75</v>
-      </c>
-      <c r="I152" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="J152" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K152" s="10" t="n"/>
-      <c r="L152" s="15">
-        <f>IF(OR(E152="",J152=""),"",(E152-J152)/E152)</f>
-        <v/>
-      </c>
-      <c r="M152" s="15" t="n"/>
-      <c r="N152" s="10" t="n"/>
-      <c r="O152" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: DebitCard | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L152" s="22" t="n"/>
+      <c r="M152" s="22" t="n"/>
     </row>
     <row r="153">
-      <c r="A153" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B153" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C153" s="5" t="inlineStr">
-        <is>
-          <t>debit card</t>
-        </is>
-      </c>
-      <c r="D153" s="8" t="n">
-        <v>500</v>
-      </c>
-      <c r="E153" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F153" s="9" t="n"/>
-      <c r="G153" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H153" s="12" t="n">
-        <v>54108.75</v>
-      </c>
-      <c r="I153" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="J153" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K153" s="10" t="n"/>
-      <c r="L153" s="15">
-        <f>IF(OR(E153="",J153=""),"",(E153-J153)/E153)</f>
-        <v/>
-      </c>
-      <c r="M153" s="15" t="n"/>
-      <c r="N153" s="10" t="n"/>
-      <c r="O153" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: DebitCard | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L153" s="22" t="n"/>
+      <c r="M153" s="22" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B154" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C154" s="5" t="inlineStr">
-        <is>
-          <t>debit card</t>
-        </is>
-      </c>
-      <c r="D154" s="8" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E154" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F154" s="9" t="n"/>
-      <c r="G154" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H154" s="12" t="n">
-        <v>108217.5</v>
-      </c>
-      <c r="I154" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J154" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K154" s="10" t="n"/>
-      <c r="L154" s="15">
-        <f>IF(OR(E154="",J154=""),"",(E154-J154)/E154)</f>
-        <v/>
-      </c>
-      <c r="M154" s="15" t="n"/>
-      <c r="N154" s="10" t="n"/>
-      <c r="O154" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: DebitCard | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L154" s="22" t="n"/>
+      <c r="M154" s="22" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B155" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C155" s="5" t="inlineStr">
-        <is>
-          <t>debit card</t>
-        </is>
-      </c>
-      <c r="D155" s="8" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E155" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F155" s="9" t="n"/>
-      <c r="G155" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H155" s="12" t="n">
-        <v>216435</v>
-      </c>
-      <c r="I155" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J155" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K155" s="10" t="n"/>
-      <c r="L155" s="15">
-        <f>IF(OR(E155="",J155=""),"",(E155-J155)/E155)</f>
-        <v/>
-      </c>
-      <c r="M155" s="15" t="n"/>
-      <c r="N155" s="10" t="n"/>
-      <c r="O155" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: DebitCard | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L155" s="22" t="n"/>
+      <c r="M155" s="22" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B156" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C156" s="5" t="inlineStr">
-        <is>
-          <t>debit card</t>
-        </is>
-      </c>
-      <c r="D156" s="8" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E156" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F156" s="9" t="n"/>
-      <c r="G156" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H156" s="12" t="n">
-        <v>541087.5</v>
-      </c>
-      <c r="I156" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J156" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K156" s="10" t="n"/>
-      <c r="L156" s="15">
-        <f>IF(OR(E156="",J156=""),"",(E156-J156)/E156)</f>
-        <v/>
-      </c>
-      <c r="M156" s="15" t="n"/>
-      <c r="N156" s="10" t="n"/>
-      <c r="O156" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: DebitCard | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L156" s="22" t="n"/>
+      <c r="M156" s="22" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B157" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C157" s="5" t="inlineStr">
-        <is>
-          <t>credit card</t>
-        </is>
-      </c>
-      <c r="D157" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="E157" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F157" s="9" t="n"/>
-      <c r="G157" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H157" s="12" t="n">
-        <v>10821.75</v>
-      </c>
-      <c r="I157" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="J157" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K157" s="10" t="n"/>
-      <c r="L157" s="15">
-        <f>IF(OR(E157="",J157=""),"",(E157-J157)/E157)</f>
-        <v/>
-      </c>
-      <c r="M157" s="15" t="n"/>
-      <c r="N157" s="10" t="n"/>
-      <c r="O157" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: CreditCard | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L157" s="22" t="n"/>
+      <c r="M157" s="22" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B158" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C158" s="5" t="inlineStr">
-        <is>
-          <t>credit card</t>
-        </is>
-      </c>
-      <c r="D158" s="8" t="n">
-        <v>500</v>
-      </c>
-      <c r="E158" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F158" s="9" t="n"/>
-      <c r="G158" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H158" s="12" t="n">
-        <v>54108.75</v>
-      </c>
-      <c r="I158" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="J158" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K158" s="10" t="n"/>
-      <c r="L158" s="15">
-        <f>IF(OR(E158="",J158=""),"",(E158-J158)/E158)</f>
-        <v/>
-      </c>
-      <c r="M158" s="15" t="n"/>
-      <c r="N158" s="10" t="n"/>
-      <c r="O158" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: CreditCard | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L158" s="22" t="n"/>
+      <c r="M158" s="22" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B159" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C159" s="5" t="inlineStr">
-        <is>
-          <t>credit card</t>
-        </is>
-      </c>
-      <c r="D159" s="8" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E159" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F159" s="9" t="n"/>
-      <c r="G159" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H159" s="12" t="n">
-        <v>108217.5</v>
-      </c>
-      <c r="I159" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J159" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K159" s="10" t="n"/>
-      <c r="L159" s="15">
-        <f>IF(OR(E159="",J159=""),"",(E159-J159)/E159)</f>
-        <v/>
-      </c>
-      <c r="M159" s="15" t="n"/>
-      <c r="N159" s="10" t="n"/>
-      <c r="O159" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: CreditCard | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L159" s="22" t="n"/>
+      <c r="M159" s="22" t="n"/>
     </row>
     <row r="160">
-      <c r="A160" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B160" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C160" s="5" t="inlineStr">
-        <is>
-          <t>credit card</t>
-        </is>
-      </c>
-      <c r="D160" s="8" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E160" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F160" s="9" t="n"/>
-      <c r="G160" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H160" s="12" t="n">
-        <v>216435</v>
-      </c>
-      <c r="I160" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J160" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K160" s="10" t="n"/>
-      <c r="L160" s="15">
-        <f>IF(OR(E160="",J160=""),"",(E160-J160)/E160)</f>
-        <v/>
-      </c>
-      <c r="M160" s="15" t="n"/>
-      <c r="N160" s="10" t="n"/>
-      <c r="O160" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: CreditCard | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L160" s="22" t="n"/>
+      <c r="M160" s="22" t="n"/>
     </row>
     <row r="161">
-      <c r="A161" s="5" t="inlineStr">
-        <is>
-          <t>XE</t>
-        </is>
-      </c>
-      <c r="B161" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C161" s="5" t="inlineStr">
-        <is>
-          <t>credit card</t>
-        </is>
-      </c>
-      <c r="D161" s="8" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E161" s="9" t="n">
-        <v>108.793</v>
-      </c>
-      <c r="F161" s="9" t="n"/>
-      <c r="G161" s="21" t="inlineStr">
-        <is>
-          <t>10:47</t>
-        </is>
-      </c>
-      <c r="H161" s="12" t="n">
-        <v>541087.5</v>
-      </c>
-      <c r="I161" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J161" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K161" s="10" t="n"/>
-      <c r="L161" s="15">
-        <f>IF(OR(E161="",J161=""),"",(E161-J161)/E161)</f>
-        <v/>
-      </c>
-      <c r="M161" s="15" t="n"/>
-      <c r="N161" s="10" t="n"/>
-      <c r="O161" s="16" t="inlineStr">
-        <is>
-          <t>XE settlement: CreditCard | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L161" s="22" t="n"/>
+      <c r="M161" s="22" t="n"/>
     </row>
     <row r="162">
       <c r="L162" s="22" t="n"/>
@@ -11217,66 +10527,6 @@
     <row r="984">
       <c r="L984" s="22" t="n"/>
       <c r="M984" s="22" t="n"/>
-    </row>
-    <row r="985">
-      <c r="L985" s="22" t="n"/>
-      <c r="M985" s="22" t="n"/>
-    </row>
-    <row r="986">
-      <c r="L986" s="22" t="n"/>
-      <c r="M986" s="22" t="n"/>
-    </row>
-    <row r="987">
-      <c r="L987" s="22" t="n"/>
-      <c r="M987" s="22" t="n"/>
-    </row>
-    <row r="988">
-      <c r="L988" s="22" t="n"/>
-      <c r="M988" s="22" t="n"/>
-    </row>
-    <row r="989">
-      <c r="L989" s="22" t="n"/>
-      <c r="M989" s="22" t="n"/>
-    </row>
-    <row r="990">
-      <c r="L990" s="22" t="n"/>
-      <c r="M990" s="22" t="n"/>
-    </row>
-    <row r="991">
-      <c r="L991" s="22" t="n"/>
-      <c r="M991" s="22" t="n"/>
-    </row>
-    <row r="992">
-      <c r="L992" s="22" t="n"/>
-      <c r="M992" s="22" t="n"/>
-    </row>
-    <row r="993">
-      <c r="L993" s="22" t="n"/>
-      <c r="M993" s="22" t="n"/>
-    </row>
-    <row r="994">
-      <c r="L994" s="22" t="n"/>
-      <c r="M994" s="22" t="n"/>
-    </row>
-    <row r="995">
-      <c r="L995" s="22" t="n"/>
-      <c r="M995" s="22" t="n"/>
-    </row>
-    <row r="996">
-      <c r="L996" s="22" t="n"/>
-      <c r="M996" s="22" t="n"/>
-    </row>
-    <row r="997">
-      <c r="L997" s="22" t="n"/>
-      <c r="M997" s="22" t="n"/>
-    </row>
-    <row r="998">
-      <c r="L998" s="22" t="n"/>
-      <c r="M998" s="22" t="n"/>
-    </row>
-    <row r="999">
-      <c r="L999" s="22" t="n"/>
-      <c r="M999" s="22" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
Scraped EUR→INR rates 2026-09-30
</commit_message>
<xml_diff>
--- a/data/EURINR_data.xlsx
+++ b/data/EURINR_data.xlsx
@@ -7177,196 +7177,2426 @@
       </c>
     </row>
     <row r="147">
-      <c r="L147" s="22" t="n"/>
-      <c r="M147" s="22" t="n"/>
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B147" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D147" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E147" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F147" s="9" t="n"/>
+      <c r="G147" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H147" s="12" t="n">
+        <v>10708</v>
+      </c>
+      <c r="I147" s="8" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="J147" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K147" s="10" t="n"/>
+      <c r="L147" s="15">
+        <f>IF(OR(E147="",J147=""),"",(E147-J147)/E147)</f>
+        <v/>
+      </c>
+      <c r="M147" s="15" t="n"/>
+      <c r="N147" s="10" t="n"/>
+      <c r="O147" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="148">
-      <c r="L148" s="22" t="n"/>
-      <c r="M148" s="22" t="n"/>
+      <c r="A148" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B148" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C148" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D148" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="E148" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F148" s="9" t="n"/>
+      <c r="G148" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H148" s="12" t="n">
+        <v>53980.62</v>
+      </c>
+      <c r="I148" s="8" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="J148" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K148" s="10" t="n"/>
+      <c r="L148" s="15">
+        <f>IF(OR(E148="",J148=""),"",(E148-J148)/E148)</f>
+        <v/>
+      </c>
+      <c r="M148" s="15" t="n"/>
+      <c r="N148" s="10" t="n"/>
+      <c r="O148" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="149">
-      <c r="L149" s="22" t="n"/>
-      <c r="M149" s="22" t="n"/>
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B149" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D149" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E149" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F149" s="9" t="n"/>
+      <c r="G149" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H149" s="12" t="n">
+        <v>108072.22</v>
+      </c>
+      <c r="I149" s="8" t="n">
+        <v>6.68</v>
+      </c>
+      <c r="J149" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K149" s="10" t="n"/>
+      <c r="L149" s="15">
+        <f>IF(OR(E149="",J149=""),"",(E149-J149)/E149)</f>
+        <v/>
+      </c>
+      <c r="M149" s="15" t="n"/>
+      <c r="N149" s="10" t="n"/>
+      <c r="O149" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="150">
-      <c r="L150" s="22" t="n"/>
-      <c r="M150" s="22" t="n"/>
+      <c r="A150" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B150" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C150" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D150" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E150" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F150" s="9" t="n"/>
+      <c r="G150" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H150" s="12" t="n">
+        <v>216253.24</v>
+      </c>
+      <c r="I150" s="8" t="n">
+        <v>12.36</v>
+      </c>
+      <c r="J150" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K150" s="10" t="n"/>
+      <c r="L150" s="15">
+        <f>IF(OR(E150="",J150=""),"",(E150-J150)/E150)</f>
+        <v/>
+      </c>
+      <c r="M150" s="15" t="n"/>
+      <c r="N150" s="10" t="n"/>
+      <c r="O150" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="151">
-      <c r="L151" s="22" t="n"/>
-      <c r="M151" s="22" t="n"/>
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B151" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D151" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E151" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F151" s="9" t="n"/>
+      <c r="G151" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H151" s="12" t="n">
+        <v>540800.66</v>
+      </c>
+      <c r="I151" s="8" t="n">
+        <v>29.36</v>
+      </c>
+      <c r="J151" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K151" s="10" t="n"/>
+      <c r="L151" s="15">
+        <f>IF(OR(E151="",J151=""),"",(E151-J151)/E151)</f>
+        <v/>
+      </c>
+      <c r="M151" s="15" t="n"/>
+      <c r="N151" s="10" t="n"/>
+      <c r="O151" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="152">
-      <c r="L152" s="22" t="n"/>
-      <c r="M152" s="22" t="n"/>
+      <c r="A152" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B152" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C152" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D152" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E152" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F152" s="9" t="n"/>
+      <c r="G152" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H152" s="12" t="n">
+        <v>10623.13</v>
+      </c>
+      <c r="I152" s="8" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="J152" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K152" s="10" t="n"/>
+      <c r="L152" s="15">
+        <f>IF(OR(E152="",J152=""),"",(E152-J152)/E152)</f>
+        <v/>
+      </c>
+      <c r="M152" s="15" t="n"/>
+      <c r="N152" s="10" t="n"/>
+      <c r="O152" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="153">
-      <c r="L153" s="22" t="n"/>
-      <c r="M153" s="22" t="n"/>
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B153" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D153" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="E153" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F153" s="9" t="n"/>
+      <c r="G153" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H153" s="12" t="n">
+        <v>53554.13</v>
+      </c>
+      <c r="I153" s="8" t="n">
+        <v>7.77</v>
+      </c>
+      <c r="J153" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K153" s="10" t="n"/>
+      <c r="L153" s="15">
+        <f>IF(OR(E153="",J153=""),"",(E153-J153)/E153)</f>
+        <v/>
+      </c>
+      <c r="M153" s="15" t="n"/>
+      <c r="N153" s="10" t="n"/>
+      <c r="O153" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="154">
-      <c r="L154" s="22" t="n"/>
-      <c r="M154" s="22" t="n"/>
+      <c r="A154" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B154" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C154" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D154" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E154" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F154" s="9" t="n"/>
+      <c r="G154" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H154" s="12" t="n">
+        <v>107220.33</v>
+      </c>
+      <c r="I154" s="8" t="n">
+        <v>14.51</v>
+      </c>
+      <c r="J154" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K154" s="10" t="n"/>
+      <c r="L154" s="15">
+        <f>IF(OR(E154="",J154=""),"",(E154-J154)/E154)</f>
+        <v/>
+      </c>
+      <c r="M154" s="15" t="n"/>
+      <c r="N154" s="10" t="n"/>
+      <c r="O154" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="155">
-      <c r="L155" s="22" t="n"/>
-      <c r="M155" s="22" t="n"/>
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B155" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D155" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E155" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F155" s="9" t="n"/>
+      <c r="G155" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H155" s="12" t="n">
+        <v>214546.19</v>
+      </c>
+      <c r="I155" s="8" t="n">
+        <v>28.05</v>
+      </c>
+      <c r="J155" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K155" s="10" t="n"/>
+      <c r="L155" s="15">
+        <f>IF(OR(E155="",J155=""),"",(E155-J155)/E155)</f>
+        <v/>
+      </c>
+      <c r="M155" s="15" t="n"/>
+      <c r="N155" s="10" t="n"/>
+      <c r="O155" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="156">
-      <c r="L156" s="22" t="n"/>
-      <c r="M156" s="22" t="n"/>
+      <c r="A156" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B156" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C156" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D156" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E156" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F156" s="9" t="n"/>
+      <c r="G156" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H156" s="12" t="n">
+        <v>536534.65</v>
+      </c>
+      <c r="I156" s="8" t="n">
+        <v>68.56999999999999</v>
+      </c>
+      <c r="J156" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K156" s="10" t="n"/>
+      <c r="L156" s="15">
+        <f>IF(OR(E156="",J156=""),"",(E156-J156)/E156)</f>
+        <v/>
+      </c>
+      <c r="M156" s="15" t="n"/>
+      <c r="N156" s="10" t="n"/>
+      <c r="O156" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="157">
-      <c r="L157" s="22" t="n"/>
-      <c r="M157" s="22" t="n"/>
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B157" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>credit card</t>
+        </is>
+      </c>
+      <c r="D157" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E157" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F157" s="9" t="n"/>
+      <c r="G157" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H157" s="12" t="n">
+        <v>10557.85</v>
+      </c>
+      <c r="I157" s="8" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="J157" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K157" s="10" t="n"/>
+      <c r="L157" s="15">
+        <f>IF(OR(E157="",J157=""),"",(E157-J157)/E157)</f>
+        <v/>
+      </c>
+      <c r="M157" s="15" t="n"/>
+      <c r="N157" s="10" t="n"/>
+      <c r="O157" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="158">
-      <c r="L158" s="22" t="n"/>
-      <c r="M158" s="22" t="n"/>
+      <c r="A158" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B158" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>credit card</t>
+        </is>
+      </c>
+      <c r="D158" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="E158" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F158" s="9" t="n"/>
+      <c r="G158" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H158" s="12" t="n">
+        <v>53227.73</v>
+      </c>
+      <c r="I158" s="8" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="J158" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K158" s="10" t="n"/>
+      <c r="L158" s="15">
+        <f>IF(OR(E158="",J158=""),"",(E158-J158)/E158)</f>
+        <v/>
+      </c>
+      <c r="M158" s="15" t="n"/>
+      <c r="N158" s="10" t="n"/>
+      <c r="O158" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="159">
-      <c r="L159" s="22" t="n"/>
-      <c r="M159" s="22" t="n"/>
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B159" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>credit card</t>
+        </is>
+      </c>
+      <c r="D159" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E159" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F159" s="9" t="n"/>
+      <c r="G159" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H159" s="12" t="n">
+        <v>106566.44</v>
+      </c>
+      <c r="I159" s="8" t="n">
+        <v>20.52</v>
+      </c>
+      <c r="J159" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K159" s="10" t="n"/>
+      <c r="L159" s="15">
+        <f>IF(OR(E159="",J159=""),"",(E159-J159)/E159)</f>
+        <v/>
+      </c>
+      <c r="M159" s="15" t="n"/>
+      <c r="N159" s="10" t="n"/>
+      <c r="O159" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="160">
-      <c r="L160" s="22" t="n"/>
-      <c r="M160" s="22" t="n"/>
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B160" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>credit card</t>
+        </is>
+      </c>
+      <c r="D160" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E160" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F160" s="9" t="n"/>
+      <c r="G160" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H160" s="12" t="n">
+        <v>213242.78</v>
+      </c>
+      <c r="I160" s="8" t="n">
+        <v>40.03</v>
+      </c>
+      <c r="J160" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K160" s="10" t="n"/>
+      <c r="L160" s="15">
+        <f>IF(OR(E160="",J160=""),"",(E160-J160)/E160)</f>
+        <v/>
+      </c>
+      <c r="M160" s="15" t="n"/>
+      <c r="N160" s="10" t="n"/>
+      <c r="O160" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="161">
-      <c r="L161" s="22" t="n"/>
-      <c r="M161" s="22" t="n"/>
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B161" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>credit card</t>
+        </is>
+      </c>
+      <c r="D161" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E161" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F161" s="9" t="n"/>
+      <c r="G161" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H161" s="12" t="n">
+        <v>533271.77</v>
+      </c>
+      <c r="I161" s="8" t="n">
+        <v>98.56</v>
+      </c>
+      <c r="J161" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="K161" s="10" t="n"/>
+      <c r="L161" s="15">
+        <f>IF(OR(E161="",J161=""),"",(E161-J161)/E161)</f>
+        <v/>
+      </c>
+      <c r="M161" s="15" t="n"/>
+      <c r="N161" s="10" t="n"/>
+      <c r="O161" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="162">
-      <c r="L162" s="22" t="n"/>
-      <c r="M162" s="22" t="n"/>
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B162" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D162" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E162" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F162" s="9" t="n"/>
+      <c r="G162" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H162" s="12" t="n">
+        <v>108217.5</v>
+      </c>
+      <c r="I162" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J162" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K162" s="10" t="n"/>
+      <c r="L162" s="15">
+        <f>IF(OR(E162="",J162=""),"",(E162-J162)/E162)</f>
+        <v/>
+      </c>
+      <c r="M162" s="15" t="n"/>
+      <c r="N162" s="10" t="n"/>
+      <c r="O162" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: BankTransfer; XE charges the fee on top, row shows €1000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="163">
-      <c r="L163" s="22" t="n"/>
-      <c r="M163" s="22" t="n"/>
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B163" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D163" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E163" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F163" s="9" t="n"/>
+      <c r="G163" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H163" s="12" t="n">
+        <v>216435</v>
+      </c>
+      <c r="I163" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J163" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K163" s="10" t="n"/>
+      <c r="L163" s="15">
+        <f>IF(OR(E163="",J163=""),"",(E163-J163)/E163)</f>
+        <v/>
+      </c>
+      <c r="M163" s="15" t="n"/>
+      <c r="N163" s="10" t="n"/>
+      <c r="O163" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: BankTransfer; XE charges the fee on top, row shows €2000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="164">
-      <c r="L164" s="22" t="n"/>
-      <c r="M164" s="22" t="n"/>
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B164" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D164" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E164" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F164" s="9" t="n"/>
+      <c r="G164" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H164" s="12" t="n">
+        <v>541087.5</v>
+      </c>
+      <c r="I164" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J164" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K164" s="10" t="n"/>
+      <c r="L164" s="15">
+        <f>IF(OR(E164="",J164=""),"",(E164-J164)/E164)</f>
+        <v/>
+      </c>
+      <c r="M164" s="15" t="n"/>
+      <c r="N164" s="10" t="n"/>
+      <c r="O164" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: BankTransfer; XE charges the fee on top, row shows €5000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="165">
-      <c r="L165" s="22" t="n"/>
-      <c r="M165" s="22" t="n"/>
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B165" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D165" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E165" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F165" s="9" t="n"/>
+      <c r="G165" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H165" s="12" t="n">
+        <v>10497.1</v>
+      </c>
+      <c r="I165" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J165" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K165" s="10" t="n"/>
+      <c r="L165" s="15">
+        <f>IF(OR(E165="",J165=""),"",(E165-J165)/E165)</f>
+        <v/>
+      </c>
+      <c r="M165" s="15" t="n"/>
+      <c r="N165" s="10" t="n"/>
+      <c r="O165" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €100 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="166">
-      <c r="L166" s="22" t="n"/>
-      <c r="M166" s="22" t="n"/>
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B166" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D166" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="E166" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F166" s="9" t="n"/>
+      <c r="G166" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H166" s="12" t="n">
+        <v>53784.1</v>
+      </c>
+      <c r="I166" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J166" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K166" s="10" t="n"/>
+      <c r="L166" s="15">
+        <f>IF(OR(E166="",J166=""),"",(E166-J166)/E166)</f>
+        <v/>
+      </c>
+      <c r="M166" s="15" t="n"/>
+      <c r="N166" s="10" t="n"/>
+      <c r="O166" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €500 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="167">
-      <c r="L167" s="22" t="n"/>
-      <c r="M167" s="22" t="n"/>
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B167" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D167" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E167" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F167" s="9" t="n"/>
+      <c r="G167" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H167" s="12" t="n">
+        <v>108217.5</v>
+      </c>
+      <c r="I167" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J167" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K167" s="10" t="n"/>
+      <c r="L167" s="15">
+        <f>IF(OR(E167="",J167=""),"",(E167-J167)/E167)</f>
+        <v/>
+      </c>
+      <c r="M167" s="15" t="n"/>
+      <c r="N167" s="10" t="n"/>
+      <c r="O167" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €1000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="168">
-      <c r="L168" s="22" t="n"/>
-      <c r="M168" s="22" t="n"/>
+      <c r="A168" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B168" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D168" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E168" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F168" s="9" t="n"/>
+      <c r="G168" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H168" s="12" t="n">
+        <v>216435</v>
+      </c>
+      <c r="I168" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J168" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K168" s="10" t="n"/>
+      <c r="L168" s="15">
+        <f>IF(OR(E168="",J168=""),"",(E168-J168)/E168)</f>
+        <v/>
+      </c>
+      <c r="M168" s="15" t="n"/>
+      <c r="N168" s="10" t="n"/>
+      <c r="O168" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €2000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="169">
-      <c r="L169" s="22" t="n"/>
-      <c r="M169" s="22" t="n"/>
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B169" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D169" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E169" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F169" s="9" t="n"/>
+      <c r="G169" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H169" s="12" t="n">
+        <v>541087.5</v>
+      </c>
+      <c r="I169" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J169" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K169" s="10" t="n"/>
+      <c r="L169" s="15">
+        <f>IF(OR(E169="",J169=""),"",(E169-J169)/E169)</f>
+        <v/>
+      </c>
+      <c r="M169" s="15" t="n"/>
+      <c r="N169" s="10" t="n"/>
+      <c r="O169" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €5000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="170">
-      <c r="L170" s="22" t="n"/>
-      <c r="M170" s="22" t="n"/>
+      <c r="A170" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B170" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>credit card</t>
+        </is>
+      </c>
+      <c r="D170" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E170" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F170" s="9" t="n"/>
+      <c r="G170" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H170" s="12" t="n">
+        <v>10497.1</v>
+      </c>
+      <c r="I170" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J170" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K170" s="10" t="n"/>
+      <c r="L170" s="15">
+        <f>IF(OR(E170="",J170=""),"",(E170-J170)/E170)</f>
+        <v/>
+      </c>
+      <c r="M170" s="15" t="n"/>
+      <c r="N170" s="10" t="n"/>
+      <c r="O170" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €100 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="171">
-      <c r="L171" s="22" t="n"/>
-      <c r="M171" s="22" t="n"/>
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B171" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>credit card</t>
+        </is>
+      </c>
+      <c r="D171" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="E171" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F171" s="9" t="n"/>
+      <c r="G171" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H171" s="12" t="n">
+        <v>53784.1</v>
+      </c>
+      <c r="I171" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J171" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K171" s="10" t="n"/>
+      <c r="L171" s="15">
+        <f>IF(OR(E171="",J171=""),"",(E171-J171)/E171)</f>
+        <v/>
+      </c>
+      <c r="M171" s="15" t="n"/>
+      <c r="N171" s="10" t="n"/>
+      <c r="O171" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €500 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="172">
-      <c r="L172" s="22" t="n"/>
-      <c r="M172" s="22" t="n"/>
+      <c r="A172" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B172" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C172" s="5" t="inlineStr">
+        <is>
+          <t>credit card</t>
+        </is>
+      </c>
+      <c r="D172" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E172" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F172" s="9" t="n"/>
+      <c r="G172" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H172" s="12" t="n">
+        <v>108217.5</v>
+      </c>
+      <c r="I172" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J172" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K172" s="10" t="n"/>
+      <c r="L172" s="15">
+        <f>IF(OR(E172="",J172=""),"",(E172-J172)/E172)</f>
+        <v/>
+      </c>
+      <c r="M172" s="15" t="n"/>
+      <c r="N172" s="10" t="n"/>
+      <c r="O172" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €1000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="173">
-      <c r="L173" s="22" t="n"/>
-      <c r="M173" s="22" t="n"/>
+      <c r="A173" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B173" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C173" s="5" t="inlineStr">
+        <is>
+          <t>credit card</t>
+        </is>
+      </c>
+      <c r="D173" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E173" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F173" s="9" t="n"/>
+      <c r="G173" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H173" s="12" t="n">
+        <v>216435</v>
+      </c>
+      <c r="I173" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J173" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K173" s="10" t="n"/>
+      <c r="L173" s="15">
+        <f>IF(OR(E173="",J173=""),"",(E173-J173)/E173)</f>
+        <v/>
+      </c>
+      <c r="M173" s="15" t="n"/>
+      <c r="N173" s="10" t="n"/>
+      <c r="O173" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €2000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="174">
-      <c r="L174" s="22" t="n"/>
-      <c r="M174" s="22" t="n"/>
+      <c r="A174" s="5" t="inlineStr">
+        <is>
+          <t>XE</t>
+        </is>
+      </c>
+      <c r="B174" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C174" s="5" t="inlineStr">
+        <is>
+          <t>credit card</t>
+        </is>
+      </c>
+      <c r="D174" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E174" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F174" s="9" t="n"/>
+      <c r="G174" s="21" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="H174" s="12" t="n">
+        <v>541087.5</v>
+      </c>
+      <c r="I174" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J174" s="9" t="n">
+        <v>108.2175</v>
+      </c>
+      <c r="K174" s="10" t="n"/>
+      <c r="L174" s="15">
+        <f>IF(OR(E174="",J174=""),"",(E174-J174)/E174)</f>
+        <v/>
+      </c>
+      <c r="M174" s="15" t="n"/>
+      <c r="N174" s="10" t="n"/>
+      <c r="O174" s="16" t="inlineStr">
+        <is>
+          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €5000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="175">
-      <c r="L175" s="22" t="n"/>
-      <c r="M175" s="22" t="n"/>
+      <c r="A175" s="5" t="inlineStr">
+        <is>
+          <t>Instarem</t>
+        </is>
+      </c>
+      <c r="B175" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C175" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D175" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E175" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F175" s="9" t="n"/>
+      <c r="G175" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H175" s="12" t="n">
+        <v>10868.22</v>
+      </c>
+      <c r="I175" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J175" s="9" t="n">
+        <v>108.0621</v>
+      </c>
+      <c r="K175" s="10" t="n">
+        <v>108.6822</v>
+      </c>
+      <c r="L175" s="15">
+        <f>IF(OR(E175="",J175=""),"",(E175-J175)/E175)</f>
+        <v/>
+      </c>
+      <c r="M175" s="15" t="n"/>
+      <c r="N175" s="10" t="n"/>
+      <c r="O175" s="16" t="inlineStr">
+        <is>
+          <t>First-transfer rate 108.6822 shown; regular rate 108.0621 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="176">
-      <c r="L176" s="22" t="n"/>
-      <c r="M176" s="22" t="n"/>
+      <c r="A176" s="5" t="inlineStr">
+        <is>
+          <t>Instarem</t>
+        </is>
+      </c>
+      <c r="B176" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C176" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D176" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="E176" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F176" s="9" t="n"/>
+      <c r="G176" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H176" s="12" t="n">
+        <v>54341.1</v>
+      </c>
+      <c r="I176" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J176" s="9" t="n">
+        <v>108.1056</v>
+      </c>
+      <c r="K176" s="10" t="n">
+        <v>108.6822</v>
+      </c>
+      <c r="L176" s="15">
+        <f>IF(OR(E176="",J176=""),"",(E176-J176)/E176)</f>
+        <v/>
+      </c>
+      <c r="M176" s="15" t="n"/>
+      <c r="N176" s="10" t="n"/>
+      <c r="O176" s="16" t="inlineStr">
+        <is>
+          <t>First-transfer rate 108.6822 shown; regular rate 108.1056 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="177">
-      <c r="L177" s="22" t="n"/>
-      <c r="M177" s="22" t="n"/>
+      <c r="A177" s="5" t="inlineStr">
+        <is>
+          <t>Instarem</t>
+        </is>
+      </c>
+      <c r="B177" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D177" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E177" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F177" s="9" t="n"/>
+      <c r="G177" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H177" s="12" t="n">
+        <v>108682.2</v>
+      </c>
+      <c r="I177" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J177" s="9" t="n">
+        <v>108.1383</v>
+      </c>
+      <c r="K177" s="10" t="n">
+        <v>108.6822</v>
+      </c>
+      <c r="L177" s="15">
+        <f>IF(OR(E177="",J177=""),"",(E177-J177)/E177)</f>
+        <v/>
+      </c>
+      <c r="M177" s="15" t="n"/>
+      <c r="N177" s="10" t="n"/>
+      <c r="O177" s="16" t="inlineStr">
+        <is>
+          <t>First-transfer rate 108.6822 shown; regular rate 108.1383 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="178">
-      <c r="L178" s="22" t="n"/>
-      <c r="M178" s="22" t="n"/>
+      <c r="A178" s="5" t="inlineStr">
+        <is>
+          <t>Instarem</t>
+        </is>
+      </c>
+      <c r="B178" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C178" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D178" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E178" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F178" s="9" t="n"/>
+      <c r="G178" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H178" s="12" t="n">
+        <v>217364.4</v>
+      </c>
+      <c r="I178" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J178" s="9" t="n">
+        <v>108.1383</v>
+      </c>
+      <c r="K178" s="10" t="n">
+        <v>108.6822</v>
+      </c>
+      <c r="L178" s="15">
+        <f>IF(OR(E178="",J178=""),"",(E178-J178)/E178)</f>
+        <v/>
+      </c>
+      <c r="M178" s="15" t="n"/>
+      <c r="N178" s="10" t="n"/>
+      <c r="O178" s="16" t="inlineStr">
+        <is>
+          <t>First-transfer rate 108.6822 shown; regular rate 108.1383 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="179">
-      <c r="L179" s="22" t="n"/>
-      <c r="M179" s="22" t="n"/>
+      <c r="A179" s="5" t="inlineStr">
+        <is>
+          <t>Instarem</t>
+        </is>
+      </c>
+      <c r="B179" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C179" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D179" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E179" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F179" s="9" t="n"/>
+      <c r="G179" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H179" s="12" t="n">
+        <v>540963</v>
+      </c>
+      <c r="I179" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J179" s="9" t="n">
+        <v>108.247</v>
+      </c>
+      <c r="K179" s="10" t="n"/>
+      <c r="L179" s="15">
+        <f>IF(OR(E179="",J179=""),"",(E179-J179)/E179)</f>
+        <v/>
+      </c>
+      <c r="M179" s="15" t="n"/>
+      <c r="N179" s="10" t="n"/>
+      <c r="O179" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="180">
-      <c r="L180" s="22" t="n"/>
-      <c r="M180" s="22" t="n"/>
+      <c r="A180" s="5" t="inlineStr">
+        <is>
+          <t>Instarem</t>
+        </is>
+      </c>
+      <c r="B180" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C180" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D180" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E180" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F180" s="9" t="n"/>
+      <c r="G180" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H180" s="12" t="n">
+        <v>10865.92</v>
+      </c>
+      <c r="I180" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J180" s="9" t="n">
+        <v>108.0393</v>
+      </c>
+      <c r="K180" s="10" t="n">
+        <v>108.6592</v>
+      </c>
+      <c r="L180" s="15">
+        <f>IF(OR(E180="",J180=""),"",(E180-J180)/E180)</f>
+        <v/>
+      </c>
+      <c r="M180" s="15" t="n"/>
+      <c r="N180" s="10" t="n"/>
+      <c r="O180" s="16" t="inlineStr">
+        <is>
+          <t>First-transfer rate 108.6592 shown; regular rate 108.0393 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="181">
-      <c r="L181" s="22" t="n"/>
-      <c r="M181" s="22" t="n"/>
+      <c r="A181" s="5" t="inlineStr">
+        <is>
+          <t>Instarem</t>
+        </is>
+      </c>
+      <c r="B181" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D181" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="E181" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F181" s="9" t="n"/>
+      <c r="G181" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H181" s="12" t="n">
+        <v>54329.6</v>
+      </c>
+      <c r="I181" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J181" s="9" t="n">
+        <v>108.0828</v>
+      </c>
+      <c r="K181" s="10" t="n">
+        <v>108.6592</v>
+      </c>
+      <c r="L181" s="15">
+        <f>IF(OR(E181="",J181=""),"",(E181-J181)/E181)</f>
+        <v/>
+      </c>
+      <c r="M181" s="15" t="n"/>
+      <c r="N181" s="10" t="n"/>
+      <c r="O181" s="16" t="inlineStr">
+        <is>
+          <t>First-transfer rate 108.6592 shown; regular rate 108.0828 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="182">
-      <c r="L182" s="22" t="n"/>
-      <c r="M182" s="22" t="n"/>
+      <c r="A182" s="5" t="inlineStr">
+        <is>
+          <t>Instarem</t>
+        </is>
+      </c>
+      <c r="B182" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C182" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D182" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E182" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F182" s="9" t="n"/>
+      <c r="G182" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H182" s="12" t="n">
+        <v>108682.2</v>
+      </c>
+      <c r="I182" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J182" s="9" t="n">
+        <v>108.1383</v>
+      </c>
+      <c r="K182" s="10" t="n">
+        <v>108.6822</v>
+      </c>
+      <c r="L182" s="15">
+        <f>IF(OR(E182="",J182=""),"",(E182-J182)/E182)</f>
+        <v/>
+      </c>
+      <c r="M182" s="15" t="n"/>
+      <c r="N182" s="10" t="n"/>
+      <c r="O182" s="16" t="inlineStr">
+        <is>
+          <t>First-transfer rate 108.6822 shown; regular rate 108.1383 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="183">
-      <c r="L183" s="22" t="n"/>
-      <c r="M183" s="22" t="n"/>
+      <c r="A183" s="5" t="inlineStr">
+        <is>
+          <t>Instarem</t>
+        </is>
+      </c>
+      <c r="B183" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C183" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D183" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E183" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F183" s="9" t="n"/>
+      <c r="G183" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H183" s="12" t="n">
+        <v>217364.4</v>
+      </c>
+      <c r="I183" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J183" s="9" t="n">
+        <v>108.1383</v>
+      </c>
+      <c r="K183" s="10" t="n">
+        <v>108.6822</v>
+      </c>
+      <c r="L183" s="15">
+        <f>IF(OR(E183="",J183=""),"",(E183-J183)/E183)</f>
+        <v/>
+      </c>
+      <c r="M183" s="15" t="n"/>
+      <c r="N183" s="10" t="n"/>
+      <c r="O183" s="16" t="inlineStr">
+        <is>
+          <t>First-transfer rate 108.6822 shown; regular rate 108.1383 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="184">
-      <c r="L184" s="22" t="n"/>
-      <c r="M184" s="22" t="n"/>
+      <c r="A184" s="5" t="inlineStr">
+        <is>
+          <t>Instarem</t>
+        </is>
+      </c>
+      <c r="B184" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>debit card</t>
+        </is>
+      </c>
+      <c r="D184" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E184" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F184" s="9" t="n"/>
+      <c r="G184" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H184" s="12" t="n">
+        <v>540963</v>
+      </c>
+      <c r="I184" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J184" s="9" t="n">
+        <v>108.247</v>
+      </c>
+      <c r="K184" s="10" t="n"/>
+      <c r="L184" s="15">
+        <f>IF(OR(E184="",J184=""),"",(E184-J184)/E184)</f>
+        <v/>
+      </c>
+      <c r="M184" s="15" t="n"/>
+      <c r="N184" s="10" t="n"/>
+      <c r="O184" s="16" t="inlineStr">
+        <is>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="185">
-      <c r="L185" s="22" t="n"/>
-      <c r="M185" s="22" t="n"/>
+      <c r="A185" s="5" t="inlineStr">
+        <is>
+          <t>Remitly</t>
+        </is>
+      </c>
+      <c r="B185" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D185" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E185" s="9" t="n">
+        <v>108.793</v>
+      </c>
+      <c r="F185" s="9" t="n"/>
+      <c r="G185" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H185" s="12" t="n">
+        <v>10913</v>
+      </c>
+      <c r="I185" s="8" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J185" s="9" t="n">
+        <v>107.98</v>
+      </c>
+      <c r="K185" s="10" t="n">
+        <v>109.13</v>
+      </c>
+      <c r="L185" s="15">
+        <f>IF(OR(E185="",J185=""),"",(E185-J185)/E185)</f>
+        <v/>
+      </c>
+      <c r="M185" s="15" t="n"/>
+      <c r="N185" s="10" t="n"/>
+      <c r="O185" s="16" t="inlineStr">
+        <is>
+          <t>New-customer rate 109.13 up to €1000 | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="186">
-      <c r="L186" s="22" t="n"/>
-      <c r="M186" s="22" t="n"/>
+      <c r="A186" s="5" t="inlineStr">
+        <is>
+          <t>Remitly</t>
+        </is>
+      </c>
+      <c r="B186" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C186" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D186" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="E186" s="9" t="n">
+        <v>108.793</v>
+      </c>
+      <c r="F186" s="9" t="n"/>
+      <c r="G186" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H186" s="12" t="n">
+        <v>54565</v>
+      </c>
+      <c r="I186" s="8" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J186" s="9" t="n">
+        <v>107.98</v>
+      </c>
+      <c r="K186" s="10" t="n">
+        <v>109.13</v>
+      </c>
+      <c r="L186" s="15">
+        <f>IF(OR(E186="",J186=""),"",(E186-J186)/E186)</f>
+        <v/>
+      </c>
+      <c r="M186" s="15" t="n"/>
+      <c r="N186" s="10" t="n"/>
+      <c r="O186" s="16" t="inlineStr">
+        <is>
+          <t>New-customer rate 109.13 up to €1000 | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="187">
-      <c r="L187" s="22" t="n"/>
-      <c r="M187" s="22" t="n"/>
+      <c r="A187" s="5" t="inlineStr">
+        <is>
+          <t>Remitly</t>
+        </is>
+      </c>
+      <c r="B187" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D187" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E187" s="9" t="n">
+        <v>108.793</v>
+      </c>
+      <c r="F187" s="9" t="n"/>
+      <c r="G187" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H187" s="12" t="n">
+        <v>109130</v>
+      </c>
+      <c r="I187" s="8" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J187" s="9" t="n">
+        <v>107.98</v>
+      </c>
+      <c r="K187" s="10" t="n">
+        <v>109.13</v>
+      </c>
+      <c r="L187" s="15">
+        <f>IF(OR(E187="",J187=""),"",(E187-J187)/E187)</f>
+        <v/>
+      </c>
+      <c r="M187" s="15" t="n"/>
+      <c r="N187" s="10" t="n"/>
+      <c r="O187" s="16" t="inlineStr">
+        <is>
+          <t>New-customer rate 109.13 up to €1000 | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="188">
-      <c r="L188" s="22" t="n"/>
-      <c r="M188" s="22" t="n"/>
+      <c r="A188" s="5" t="inlineStr">
+        <is>
+          <t>Remitly</t>
+        </is>
+      </c>
+      <c r="B188" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C188" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D188" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E188" s="9" t="n">
+        <v>108.793</v>
+      </c>
+      <c r="F188" s="9" t="n"/>
+      <c r="G188" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H188" s="12" t="n">
+        <v>217110</v>
+      </c>
+      <c r="I188" s="8" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J188" s="9" t="n">
+        <v>107.98</v>
+      </c>
+      <c r="K188" s="10" t="n"/>
+      <c r="L188" s="15">
+        <f>IF(OR(E188="",J188=""),"",(E188-J188)/E188)</f>
+        <v/>
+      </c>
+      <c r="M188" s="15" t="n"/>
+      <c r="N188" s="10" t="n"/>
+      <c r="O188" s="16" t="inlineStr">
+        <is>
+          <t>New-customer rate 109.13 up to €1000 | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="189">
-      <c r="L189" s="22" t="n"/>
-      <c r="M189" s="22" t="n"/>
+      <c r="A189" s="5" t="inlineStr">
+        <is>
+          <t>Remitly</t>
+        </is>
+      </c>
+      <c r="B189" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D189" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E189" s="9" t="n">
+        <v>108.793</v>
+      </c>
+      <c r="F189" s="9" t="n"/>
+      <c r="G189" s="21" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="H189" s="12" t="n">
+        <v>541050</v>
+      </c>
+      <c r="I189" s="8" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J189" s="9" t="n">
+        <v>107.98</v>
+      </c>
+      <c r="K189" s="10" t="n"/>
+      <c r="L189" s="15">
+        <f>IF(OR(E189="",J189=""),"",(E189-J189)/E189)</f>
+        <v/>
+      </c>
+      <c r="M189" s="15" t="n"/>
+      <c r="N189" s="10" t="n"/>
+      <c r="O189" s="16" t="inlineStr">
+        <is>
+          <t>New-customer rate 109.13 up to €1000 | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="190">
-      <c r="L190" s="22" t="n"/>
-      <c r="M190" s="22" t="n"/>
+      <c r="A190" s="5" t="inlineStr">
+        <is>
+          <t>Skrill</t>
+        </is>
+      </c>
+      <c r="B190" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C190" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D190" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E190" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F190" s="9" t="n"/>
+      <c r="G190" s="21" t="inlineStr">
+        <is>
+          <t>10:52</t>
+        </is>
+      </c>
+      <c r="H190" s="12" t="n">
+        <v>10821.77</v>
+      </c>
+      <c r="I190" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J190" s="9" t="n">
+        <v>108.2177</v>
+      </c>
+      <c r="K190" s="10" t="n"/>
+      <c r="L190" s="15">
+        <f>IF(OR(E190="",J190=""),"",(E190-J190)/E190)</f>
+        <v/>
+      </c>
+      <c r="M190" s="15" t="n"/>
+      <c r="N190" s="10" t="n"/>
+      <c r="O190" s="16" t="inlineStr">
+        <is>
+          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="191">
-      <c r="L191" s="22" t="n"/>
-      <c r="M191" s="22" t="n"/>
+      <c r="A191" s="5" t="inlineStr">
+        <is>
+          <t>Skrill</t>
+        </is>
+      </c>
+      <c r="B191" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D191" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="E191" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F191" s="9" t="n"/>
+      <c r="G191" s="21" t="inlineStr">
+        <is>
+          <t>10:52</t>
+        </is>
+      </c>
+      <c r="H191" s="12" t="n">
+        <v>54108.87</v>
+      </c>
+      <c r="I191" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J191" s="9" t="n">
+        <v>108.2177</v>
+      </c>
+      <c r="K191" s="10" t="n"/>
+      <c r="L191" s="15">
+        <f>IF(OR(E191="",J191=""),"",(E191-J191)/E191)</f>
+        <v/>
+      </c>
+      <c r="M191" s="15" t="n"/>
+      <c r="N191" s="10" t="n"/>
+      <c r="O191" s="16" t="inlineStr">
+        <is>
+          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="192">
-      <c r="L192" s="22" t="n"/>
-      <c r="M192" s="22" t="n"/>
+      <c r="A192" s="5" t="inlineStr">
+        <is>
+          <t>Skrill</t>
+        </is>
+      </c>
+      <c r="B192" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C192" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D192" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E192" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F192" s="9" t="n"/>
+      <c r="G192" s="21" t="inlineStr">
+        <is>
+          <t>10:52</t>
+        </is>
+      </c>
+      <c r="H192" s="12" t="n">
+        <v>108217.74</v>
+      </c>
+      <c r="I192" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J192" s="9" t="n">
+        <v>108.2177</v>
+      </c>
+      <c r="K192" s="10" t="n"/>
+      <c r="L192" s="15">
+        <f>IF(OR(E192="",J192=""),"",(E192-J192)/E192)</f>
+        <v/>
+      </c>
+      <c r="M192" s="15" t="n"/>
+      <c r="N192" s="10" t="n"/>
+      <c r="O192" s="16" t="inlineStr">
+        <is>
+          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="193">
-      <c r="L193" s="22" t="n"/>
-      <c r="M193" s="22" t="n"/>
+      <c r="A193" s="5" t="inlineStr">
+        <is>
+          <t>Skrill</t>
+        </is>
+      </c>
+      <c r="B193" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D193" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E193" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F193" s="9" t="n"/>
+      <c r="G193" s="21" t="inlineStr">
+        <is>
+          <t>10:52</t>
+        </is>
+      </c>
+      <c r="H193" s="12" t="n">
+        <v>216435.47</v>
+      </c>
+      <c r="I193" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J193" s="9" t="n">
+        <v>108.2177</v>
+      </c>
+      <c r="K193" s="10" t="n"/>
+      <c r="L193" s="15">
+        <f>IF(OR(E193="",J193=""),"",(E193-J193)/E193)</f>
+        <v/>
+      </c>
+      <c r="M193" s="15" t="n"/>
+      <c r="N193" s="10" t="n"/>
+      <c r="O193" s="16" t="inlineStr">
+        <is>
+          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="194">
-      <c r="L194" s="22" t="n"/>
-      <c r="M194" s="22" t="n"/>
+      <c r="A194" s="5" t="inlineStr">
+        <is>
+          <t>Skrill</t>
+        </is>
+      </c>
+      <c r="B194" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C194" s="5" t="inlineStr">
+        <is>
+          <t>bank transfer</t>
+        </is>
+      </c>
+      <c r="D194" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E194" s="9" t="n">
+        <v>108.799</v>
+      </c>
+      <c r="F194" s="9" t="n"/>
+      <c r="G194" s="21" t="inlineStr">
+        <is>
+          <t>10:52</t>
+        </is>
+      </c>
+      <c r="H194" s="12" t="n">
+        <v>541088.6800000001</v>
+      </c>
+      <c r="I194" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J194" s="9" t="n">
+        <v>108.2177</v>
+      </c>
+      <c r="K194" s="10" t="n"/>
+      <c r="L194" s="15">
+        <f>IF(OR(E194="",J194=""),"",(E194-J194)/E194)</f>
+        <v/>
+      </c>
+      <c r="M194" s="15" t="n"/>
+      <c r="N194" s="10" t="n"/>
+      <c r="O194" s="16" t="inlineStr">
+        <is>
+          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="L195" s="22" t="n"/>
@@ -10533,7 +12763,7 @@
     <dataValidation sqref="A2:A131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>#REF!</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C161" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C194" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"bank transfer,debit card,credit card"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Move collector into a Google Apps Script; live provider quotes only
- apps-script/Code.gs: runs inside the Google Sheet on a Mon/Thu trigger,
  fetches Wise, XE, Instarem and Remitly from their own calculators, fills
  the Google Rate column from GOOGLEFINANCE, and writes a Run log listing
  providers to fill manually (failed ones, plus Skrill, Revolut, ScopeX)
- Drop Wise comparison data as a source and remove the Skrill rows it produced
- Remove the GitHub Actions scraper; the sheet is now the data store

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018ogxhrLjz2PWd89TeAujLA
</commit_message>
<xml_diff>
--- a/data/EURINR_data.xlsx
+++ b/data/EURINR_data.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O984"/>
+  <dimension ref="A1:O974"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="167.25" customWidth="1" style="23" min="15" max="15"/>
@@ -9351,7 +9351,7 @@
     <row r="190">
       <c r="A190" s="5" t="inlineStr">
         <is>
-          <t>Skrill</t>
+          <t>Wise</t>
         </is>
       </c>
       <c r="B190" s="11" t="inlineStr">
@@ -9368,22 +9368,22 @@
         <v>100</v>
       </c>
       <c r="E190" s="9" t="n">
-        <v>108.799</v>
+        <v>108.881</v>
       </c>
       <c r="F190" s="9" t="n"/>
       <c r="G190" s="21" t="inlineStr">
         <is>
-          <t>10:52</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="H190" s="12" t="n">
-        <v>10821.77</v>
+        <v>10716.07</v>
       </c>
       <c r="I190" s="8" t="n">
-        <v>0</v>
+        <v>1.58</v>
       </c>
       <c r="J190" s="9" t="n">
-        <v>108.2177</v>
+        <v>108.881</v>
       </c>
       <c r="K190" s="10" t="n"/>
       <c r="L190" s="15">
@@ -9394,14 +9394,14 @@
       <c r="N190" s="10" t="n"/>
       <c r="O190" s="16" t="inlineStr">
         <is>
-          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="5" t="inlineStr">
         <is>
-          <t>Skrill</t>
+          <t>Wise</t>
         </is>
       </c>
       <c r="B191" s="11" t="inlineStr">
@@ -9418,22 +9418,22 @@
         <v>500</v>
       </c>
       <c r="E191" s="9" t="n">
-        <v>108.799</v>
+        <v>108.881</v>
       </c>
       <c r="F191" s="9" t="n"/>
       <c r="G191" s="21" t="inlineStr">
         <is>
-          <t>10:52</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="H191" s="12" t="n">
-        <v>54108.87</v>
+        <v>54021.31</v>
       </c>
       <c r="I191" s="8" t="n">
-        <v>0</v>
+        <v>3.85</v>
       </c>
       <c r="J191" s="9" t="n">
-        <v>108.2177</v>
+        <v>108.881</v>
       </c>
       <c r="K191" s="10" t="n"/>
       <c r="L191" s="15">
@@ -9444,14 +9444,14 @@
       <c r="N191" s="10" t="n"/>
       <c r="O191" s="16" t="inlineStr">
         <is>
-          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="5" t="inlineStr">
         <is>
-          <t>Skrill</t>
+          <t>Wise</t>
         </is>
       </c>
       <c r="B192" s="11" t="inlineStr">
@@ -9468,22 +9468,22 @@
         <v>1000</v>
       </c>
       <c r="E192" s="9" t="n">
-        <v>108.799</v>
+        <v>108.881</v>
       </c>
       <c r="F192" s="9" t="n"/>
       <c r="G192" s="21" t="inlineStr">
         <is>
-          <t>10:52</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="H192" s="12" t="n">
-        <v>108217.74</v>
+        <v>108153.67</v>
       </c>
       <c r="I192" s="8" t="n">
-        <v>0</v>
+        <v>6.68</v>
       </c>
       <c r="J192" s="9" t="n">
-        <v>108.2177</v>
+        <v>108.881</v>
       </c>
       <c r="K192" s="10" t="n"/>
       <c r="L192" s="15">
@@ -9494,14 +9494,14 @@
       <c r="N192" s="10" t="n"/>
       <c r="O192" s="16" t="inlineStr">
         <is>
-          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="5" t="inlineStr">
         <is>
-          <t>Skrill</t>
+          <t>Wise</t>
         </is>
       </c>
       <c r="B193" s="11" t="inlineStr">
@@ -9518,22 +9518,22 @@
         <v>2000</v>
       </c>
       <c r="E193" s="9" t="n">
-        <v>108.799</v>
+        <v>108.881</v>
       </c>
       <c r="F193" s="9" t="n"/>
       <c r="G193" s="21" t="inlineStr">
         <is>
-          <t>10:52</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="H193" s="12" t="n">
-        <v>216435.47</v>
+        <v>216416.23</v>
       </c>
       <c r="I193" s="8" t="n">
-        <v>0</v>
+        <v>12.36</v>
       </c>
       <c r="J193" s="9" t="n">
-        <v>108.2177</v>
+        <v>108.881</v>
       </c>
       <c r="K193" s="10" t="n"/>
       <c r="L193" s="15">
@@ -9544,14 +9544,14 @@
       <c r="N193" s="10" t="n"/>
       <c r="O193" s="16" t="inlineStr">
         <is>
-          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="5" t="inlineStr">
         <is>
-          <t>Skrill</t>
+          <t>Wise</t>
         </is>
       </c>
       <c r="B194" s="11" t="inlineStr">
@@ -9568,22 +9568,22 @@
         <v>5000</v>
       </c>
       <c r="E194" s="9" t="n">
-        <v>108.799</v>
+        <v>108.881</v>
       </c>
       <c r="F194" s="9" t="n"/>
       <c r="G194" s="21" t="inlineStr">
         <is>
-          <t>10:52</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="H194" s="12" t="n">
-        <v>541088.6800000001</v>
+        <v>541208.25</v>
       </c>
       <c r="I194" s="8" t="n">
-        <v>0</v>
+        <v>29.36</v>
       </c>
       <c r="J194" s="9" t="n">
-        <v>108.2177</v>
+        <v>108.881</v>
       </c>
       <c r="K194" s="10" t="n"/>
       <c r="L194" s="15">
@@ -9594,7 +9594,7 @@
       <c r="N194" s="10" t="n"/>
       <c r="O194" s="16" t="inlineStr">
         <is>
-          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
@@ -9611,7 +9611,7 @@
       </c>
       <c r="C195" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D195" s="8" t="n">
@@ -9627,10 +9627,10 @@
         </is>
       </c>
       <c r="H195" s="12" t="n">
-        <v>10716.07</v>
+        <v>10631.14</v>
       </c>
       <c r="I195" s="8" t="n">
-        <v>1.58</v>
+        <v>2.36</v>
       </c>
       <c r="J195" s="9" t="n">
         <v>108.881</v>
@@ -9661,7 +9661,7 @@
       </c>
       <c r="C196" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D196" s="8" t="n">
@@ -9677,10 +9677,10 @@
         </is>
       </c>
       <c r="H196" s="12" t="n">
-        <v>54021.31</v>
+        <v>53594.49</v>
       </c>
       <c r="I196" s="8" t="n">
-        <v>3.85</v>
+        <v>7.77</v>
       </c>
       <c r="J196" s="9" t="n">
         <v>108.881</v>
@@ -9711,7 +9711,7 @@
       </c>
       <c r="C197" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D197" s="8" t="n">
@@ -9727,10 +9727,10 @@
         </is>
       </c>
       <c r="H197" s="12" t="n">
-        <v>108153.67</v>
+        <v>107301.14</v>
       </c>
       <c r="I197" s="8" t="n">
-        <v>6.68</v>
+        <v>14.51</v>
       </c>
       <c r="J197" s="9" t="n">
         <v>108.881</v>
@@ -9761,7 +9761,7 @@
       </c>
       <c r="C198" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D198" s="8" t="n">
@@ -9777,10 +9777,10 @@
         </is>
       </c>
       <c r="H198" s="12" t="n">
-        <v>216416.23</v>
+        <v>214707.89</v>
       </c>
       <c r="I198" s="8" t="n">
-        <v>12.36</v>
+        <v>28.05</v>
       </c>
       <c r="J198" s="9" t="n">
         <v>108.881</v>
@@ -9811,7 +9811,7 @@
       </c>
       <c r="C199" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D199" s="8" t="n">
@@ -9827,10 +9827,10 @@
         </is>
       </c>
       <c r="H199" s="12" t="n">
-        <v>541208.25</v>
+        <v>536939.03</v>
       </c>
       <c r="I199" s="8" t="n">
-        <v>29.36</v>
+        <v>68.56999999999999</v>
       </c>
       <c r="J199" s="9" t="n">
         <v>108.881</v>
@@ -9861,7 +9861,7 @@
       </c>
       <c r="C200" s="5" t="inlineStr">
         <is>
-          <t>debit card</t>
+          <t>credit card</t>
         </is>
       </c>
       <c r="D200" s="8" t="n">
@@ -9877,10 +9877,10 @@
         </is>
       </c>
       <c r="H200" s="12" t="n">
-        <v>10631.14</v>
+        <v>10565.81</v>
       </c>
       <c r="I200" s="8" t="n">
-        <v>2.36</v>
+        <v>2.96</v>
       </c>
       <c r="J200" s="9" t="n">
         <v>108.881</v>
@@ -9911,7 +9911,7 @@
       </c>
       <c r="C201" s="5" t="inlineStr">
         <is>
-          <t>debit card</t>
+          <t>credit card</t>
         </is>
       </c>
       <c r="D201" s="8" t="n">
@@ -9927,10 +9927,10 @@
         </is>
       </c>
       <c r="H201" s="12" t="n">
-        <v>53594.49</v>
+        <v>53267.85</v>
       </c>
       <c r="I201" s="8" t="n">
-        <v>7.77</v>
+        <v>10.77</v>
       </c>
       <c r="J201" s="9" t="n">
         <v>108.881</v>
@@ -9961,7 +9961,7 @@
       </c>
       <c r="C202" s="5" t="inlineStr">
         <is>
-          <t>debit card</t>
+          <t>credit card</t>
         </is>
       </c>
       <c r="D202" s="8" t="n">
@@ -9977,10 +9977,10 @@
         </is>
       </c>
       <c r="H202" s="12" t="n">
-        <v>107301.14</v>
+        <v>106646.76</v>
       </c>
       <c r="I202" s="8" t="n">
-        <v>14.51</v>
+        <v>20.52</v>
       </c>
       <c r="J202" s="9" t="n">
         <v>108.881</v>
@@ -10011,7 +10011,7 @@
       </c>
       <c r="C203" s="5" t="inlineStr">
         <is>
-          <t>debit card</t>
+          <t>credit card</t>
         </is>
       </c>
       <c r="D203" s="8" t="n">
@@ -10027,10 +10027,10 @@
         </is>
       </c>
       <c r="H203" s="12" t="n">
-        <v>214707.89</v>
+        <v>213403.49</v>
       </c>
       <c r="I203" s="8" t="n">
-        <v>28.05</v>
+        <v>40.03</v>
       </c>
       <c r="J203" s="9" t="n">
         <v>108.881</v>
@@ -10061,7 +10061,7 @@
       </c>
       <c r="C204" s="5" t="inlineStr">
         <is>
-          <t>debit card</t>
+          <t>credit card</t>
         </is>
       </c>
       <c r="D204" s="8" t="n">
@@ -10077,10 +10077,10 @@
         </is>
       </c>
       <c r="H204" s="12" t="n">
-        <v>536939.03</v>
+        <v>533673.6899999999</v>
       </c>
       <c r="I204" s="8" t="n">
-        <v>68.56999999999999</v>
+        <v>98.56</v>
       </c>
       <c r="J204" s="9" t="n">
         <v>108.881</v>
@@ -10101,7 +10101,7 @@
     <row r="205">
       <c r="A205" s="5" t="inlineStr">
         <is>
-          <t>Wise</t>
+          <t>XE</t>
         </is>
       </c>
       <c r="B205" s="11" t="inlineStr">
@@ -10111,11 +10111,11 @@
       </c>
       <c r="C205" s="5" t="inlineStr">
         <is>
-          <t>credit card</t>
+          <t>bank transfer</t>
         </is>
       </c>
       <c r="D205" s="8" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="E205" s="9" t="n">
         <v>108.881</v>
@@ -10127,13 +10127,13 @@
         </is>
       </c>
       <c r="H205" s="12" t="n">
-        <v>10565.81</v>
+        <v>108217.5</v>
       </c>
       <c r="I205" s="8" t="n">
-        <v>2.96</v>
+        <v>0</v>
       </c>
       <c r="J205" s="9" t="n">
-        <v>108.881</v>
+        <v>108.2175</v>
       </c>
       <c r="K205" s="10" t="n"/>
       <c r="L205" s="15">
@@ -10144,14 +10144,14 @@
       <c r="N205" s="10" t="n"/>
       <c r="O205" s="16" t="inlineStr">
         <is>
-          <t>Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: BankTransfer; XE charges the fee on top, row shows €1000 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="5" t="inlineStr">
         <is>
-          <t>Wise</t>
+          <t>XE</t>
         </is>
       </c>
       <c r="B206" s="11" t="inlineStr">
@@ -10161,11 +10161,11 @@
       </c>
       <c r="C206" s="5" t="inlineStr">
         <is>
-          <t>credit card</t>
+          <t>bank transfer</t>
         </is>
       </c>
       <c r="D206" s="8" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="E206" s="9" t="n">
         <v>108.881</v>
@@ -10177,13 +10177,13 @@
         </is>
       </c>
       <c r="H206" s="12" t="n">
-        <v>53267.85</v>
+        <v>216435</v>
       </c>
       <c r="I206" s="8" t="n">
-        <v>10.77</v>
+        <v>0</v>
       </c>
       <c r="J206" s="9" t="n">
-        <v>108.881</v>
+        <v>108.2175</v>
       </c>
       <c r="K206" s="10" t="n"/>
       <c r="L206" s="15">
@@ -10194,14 +10194,14 @@
       <c r="N206" s="10" t="n"/>
       <c r="O206" s="16" t="inlineStr">
         <is>
-          <t>Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: BankTransfer; XE charges the fee on top, row shows €2000 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="5" t="inlineStr">
         <is>
-          <t>Wise</t>
+          <t>XE</t>
         </is>
       </c>
       <c r="B207" s="11" t="inlineStr">
@@ -10211,11 +10211,11 @@
       </c>
       <c r="C207" s="5" t="inlineStr">
         <is>
-          <t>credit card</t>
+          <t>bank transfer</t>
         </is>
       </c>
       <c r="D207" s="8" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="E207" s="9" t="n">
         <v>108.881</v>
@@ -10227,13 +10227,13 @@
         </is>
       </c>
       <c r="H207" s="12" t="n">
-        <v>106646.76</v>
+        <v>541087.5</v>
       </c>
       <c r="I207" s="8" t="n">
-        <v>20.52</v>
+        <v>0</v>
       </c>
       <c r="J207" s="9" t="n">
-        <v>108.881</v>
+        <v>108.2175</v>
       </c>
       <c r="K207" s="10" t="n"/>
       <c r="L207" s="15">
@@ -10244,14 +10244,14 @@
       <c r="N207" s="10" t="n"/>
       <c r="O207" s="16" t="inlineStr">
         <is>
-          <t>Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: BankTransfer; XE charges the fee on top, row shows €5000 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="5" t="inlineStr">
         <is>
-          <t>Wise</t>
+          <t>XE</t>
         </is>
       </c>
       <c r="B208" s="11" t="inlineStr">
@@ -10261,11 +10261,11 @@
       </c>
       <c r="C208" s="5" t="inlineStr">
         <is>
-          <t>credit card</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D208" s="8" t="n">
-        <v>2000</v>
+        <v>100</v>
       </c>
       <c r="E208" s="9" t="n">
         <v>108.881</v>
@@ -10277,13 +10277,13 @@
         </is>
       </c>
       <c r="H208" s="12" t="n">
-        <v>213403.49</v>
+        <v>10497.1</v>
       </c>
       <c r="I208" s="8" t="n">
-        <v>40.03</v>
+        <v>3</v>
       </c>
       <c r="J208" s="9" t="n">
-        <v>108.881</v>
+        <v>108.2175</v>
       </c>
       <c r="K208" s="10" t="n"/>
       <c r="L208" s="15">
@@ -10294,14 +10294,14 @@
       <c r="N208" s="10" t="n"/>
       <c r="O208" s="16" t="inlineStr">
         <is>
-          <t>Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €100 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="5" t="inlineStr">
         <is>
-          <t>Wise</t>
+          <t>XE</t>
         </is>
       </c>
       <c r="B209" s="11" t="inlineStr">
@@ -10311,11 +10311,11 @@
       </c>
       <c r="C209" s="5" t="inlineStr">
         <is>
-          <t>credit card</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D209" s="8" t="n">
-        <v>5000</v>
+        <v>500</v>
       </c>
       <c r="E209" s="9" t="n">
         <v>108.881</v>
@@ -10327,13 +10327,13 @@
         </is>
       </c>
       <c r="H209" s="12" t="n">
-        <v>533673.6899999999</v>
+        <v>53784.1</v>
       </c>
       <c r="I209" s="8" t="n">
-        <v>98.56</v>
+        <v>3</v>
       </c>
       <c r="J209" s="9" t="n">
-        <v>108.881</v>
+        <v>108.2175</v>
       </c>
       <c r="K209" s="10" t="n"/>
       <c r="L209" s="15">
@@ -10344,7 +10344,7 @@
       <c r="N209" s="10" t="n"/>
       <c r="O209" s="16" t="inlineStr">
         <is>
-          <t>Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €500 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
@@ -10361,7 +10361,7 @@
       </c>
       <c r="C210" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D210" s="8" t="n">
@@ -10394,7 +10394,7 @@
       <c r="N210" s="10" t="n"/>
       <c r="O210" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: BankTransfer; XE charges the fee on top, row shows €1000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €1000 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
@@ -10411,7 +10411,7 @@
       </c>
       <c r="C211" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D211" s="8" t="n">
@@ -10444,7 +10444,7 @@
       <c r="N211" s="10" t="n"/>
       <c r="O211" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: BankTransfer; XE charges the fee on top, row shows €2000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €2000 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
@@ -10461,7 +10461,7 @@
       </c>
       <c r="C212" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D212" s="8" t="n">
@@ -10494,7 +10494,7 @@
       <c r="N212" s="10" t="n"/>
       <c r="O212" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: BankTransfer; XE charges the fee on top, row shows €5000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €5000 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
@@ -10511,7 +10511,7 @@
       </c>
       <c r="C213" s="5" t="inlineStr">
         <is>
-          <t>debit card</t>
+          <t>credit card</t>
         </is>
       </c>
       <c r="D213" s="8" t="n">
@@ -10544,7 +10544,7 @@
       <c r="N213" s="10" t="n"/>
       <c r="O213" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €100 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €100 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
@@ -10561,7 +10561,7 @@
       </c>
       <c r="C214" s="5" t="inlineStr">
         <is>
-          <t>debit card</t>
+          <t>credit card</t>
         </is>
       </c>
       <c r="D214" s="8" t="n">
@@ -10594,7 +10594,7 @@
       <c r="N214" s="10" t="n"/>
       <c r="O214" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €500 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €500 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
@@ -10611,7 +10611,7 @@
       </c>
       <c r="C215" s="5" t="inlineStr">
         <is>
-          <t>debit card</t>
+          <t>credit card</t>
         </is>
       </c>
       <c r="D215" s="8" t="n">
@@ -10644,7 +10644,7 @@
       <c r="N215" s="10" t="n"/>
       <c r="O215" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €1000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €1000 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
@@ -10661,7 +10661,7 @@
       </c>
       <c r="C216" s="5" t="inlineStr">
         <is>
-          <t>debit card</t>
+          <t>credit card</t>
         </is>
       </c>
       <c r="D216" s="8" t="n">
@@ -10694,7 +10694,7 @@
       <c r="N216" s="10" t="n"/>
       <c r="O216" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €2000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €2000 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
@@ -10711,7 +10711,7 @@
       </c>
       <c r="C217" s="5" t="inlineStr">
         <is>
-          <t>debit card</t>
+          <t>credit card</t>
         </is>
       </c>
       <c r="D217" s="8" t="n">
@@ -10744,14 +10744,14 @@
       <c r="N217" s="10" t="n"/>
       <c r="O217" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: DebitCard; XE charges the fee on top, row shows €5000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €5000 total paid | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="5" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>Instarem</t>
         </is>
       </c>
       <c r="B218" s="11" t="inlineStr">
@@ -10761,31 +10761,33 @@
       </c>
       <c r="C218" s="5" t="inlineStr">
         <is>
-          <t>credit card</t>
+          <t>bank transfer</t>
         </is>
       </c>
       <c r="D218" s="8" t="n">
         <v>100</v>
       </c>
       <c r="E218" s="9" t="n">
-        <v>108.881</v>
+        <v>108.885</v>
       </c>
       <c r="F218" s="9" t="n"/>
       <c r="G218" s="21" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="H218" s="12" t="n">
-        <v>10497.1</v>
+        <v>10875.21</v>
       </c>
       <c r="I218" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J218" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K218" s="10" t="n"/>
+        <v>108.1316</v>
+      </c>
+      <c r="K218" s="10" t="n">
+        <v>108.7521</v>
+      </c>
       <c r="L218" s="15">
         <f>IF(OR(E218="",J218=""),"",(E218-J218)/E218)</f>
         <v/>
@@ -10794,14 +10796,14 @@
       <c r="N218" s="10" t="n"/>
       <c r="O218" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €100 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>First-transfer rate 108.7521 shown; regular rate 108.1316 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="5" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>Instarem</t>
         </is>
       </c>
       <c r="B219" s="11" t="inlineStr">
@@ -10811,31 +10813,33 @@
       </c>
       <c r="C219" s="5" t="inlineStr">
         <is>
-          <t>credit card</t>
+          <t>bank transfer</t>
         </is>
       </c>
       <c r="D219" s="8" t="n">
         <v>500</v>
       </c>
       <c r="E219" s="9" t="n">
-        <v>108.881</v>
+        <v>108.885</v>
       </c>
       <c r="F219" s="9" t="n"/>
       <c r="G219" s="21" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="H219" s="12" t="n">
-        <v>53784.1</v>
+        <v>54376.05</v>
       </c>
       <c r="I219" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J219" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K219" s="10" t="n"/>
+        <v>108.1752</v>
+      </c>
+      <c r="K219" s="10" t="n">
+        <v>108.7521</v>
+      </c>
       <c r="L219" s="15">
         <f>IF(OR(E219="",J219=""),"",(E219-J219)/E219)</f>
         <v/>
@@ -10844,14 +10848,14 @@
       <c r="N219" s="10" t="n"/>
       <c r="O219" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €500 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>First-transfer rate 108.7521 shown; regular rate 108.1752 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="5" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>Instarem</t>
         </is>
       </c>
       <c r="B220" s="11" t="inlineStr">
@@ -10861,31 +10865,33 @@
       </c>
       <c r="C220" s="5" t="inlineStr">
         <is>
-          <t>credit card</t>
+          <t>bank transfer</t>
         </is>
       </c>
       <c r="D220" s="8" t="n">
         <v>1000</v>
       </c>
       <c r="E220" s="9" t="n">
-        <v>108.881</v>
+        <v>108.885</v>
       </c>
       <c r="F220" s="9" t="n"/>
       <c r="G220" s="21" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="H220" s="12" t="n">
-        <v>108217.5</v>
+        <v>108752.1</v>
       </c>
       <c r="I220" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J220" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K220" s="10" t="n"/>
+        <v>108.2078</v>
+      </c>
+      <c r="K220" s="10" t="n">
+        <v>108.7521</v>
+      </c>
       <c r="L220" s="15">
         <f>IF(OR(E220="",J220=""),"",(E220-J220)/E220)</f>
         <v/>
@@ -10894,14 +10900,14 @@
       <c r="N220" s="10" t="n"/>
       <c r="O220" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €1000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>First-transfer rate 108.7521 shown; regular rate 108.2078 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="5" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>Instarem</t>
         </is>
       </c>
       <c r="B221" s="11" t="inlineStr">
@@ -10911,31 +10917,33 @@
       </c>
       <c r="C221" s="5" t="inlineStr">
         <is>
-          <t>credit card</t>
+          <t>bank transfer</t>
         </is>
       </c>
       <c r="D221" s="8" t="n">
         <v>2000</v>
       </c>
       <c r="E221" s="9" t="n">
-        <v>108.881</v>
+        <v>108.885</v>
       </c>
       <c r="F221" s="9" t="n"/>
       <c r="G221" s="21" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="H221" s="12" t="n">
-        <v>216435</v>
+        <v>217504.2</v>
       </c>
       <c r="I221" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J221" s="9" t="n">
-        <v>108.2175</v>
-      </c>
-      <c r="K221" s="10" t="n"/>
+        <v>108.2078</v>
+      </c>
+      <c r="K221" s="10" t="n">
+        <v>108.7521</v>
+      </c>
       <c r="L221" s="15">
         <f>IF(OR(E221="",J221=""),"",(E221-J221)/E221)</f>
         <v/>
@@ -10944,14 +10952,14 @@
       <c r="N221" s="10" t="n"/>
       <c r="O221" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €2000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>First-transfer rate 108.7521 shown; regular rate 108.2078 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="5" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>Instarem</t>
         </is>
       </c>
       <c r="B222" s="11" t="inlineStr">
@@ -10961,29 +10969,29 @@
       </c>
       <c r="C222" s="5" t="inlineStr">
         <is>
-          <t>credit card</t>
+          <t>bank transfer</t>
         </is>
       </c>
       <c r="D222" s="8" t="n">
         <v>5000</v>
       </c>
       <c r="E222" s="9" t="n">
-        <v>108.881</v>
+        <v>108.885</v>
       </c>
       <c r="F222" s="9" t="n"/>
       <c r="G222" s="21" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="H222" s="12" t="n">
-        <v>541087.5</v>
+        <v>541311.5</v>
       </c>
       <c r="I222" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J222" s="9" t="n">
-        <v>108.2175</v>
+        <v>108.3167</v>
       </c>
       <c r="K222" s="10" t="n"/>
       <c r="L222" s="15">
@@ -10994,7 +11002,7 @@
       <c r="N222" s="10" t="n"/>
       <c r="O222" s="16" t="inlineStr">
         <is>
-          <t>XE settlement: CreditCard; XE charges the fee on top, row shows €5000 total paid | Auto-scraped; mid rate = Wise live mid</t>
+          <t>Auto-scraped; mid rate = Wise live mid</t>
         </is>
       </c>
     </row>
@@ -11011,7 +11019,7 @@
       </c>
       <c r="C223" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D223" s="8" t="n">
@@ -11063,7 +11071,7 @@
       </c>
       <c r="C224" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D224" s="8" t="n">
@@ -11115,7 +11123,7 @@
       </c>
       <c r="C225" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D225" s="8" t="n">
@@ -11167,7 +11175,7 @@
       </c>
       <c r="C226" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D226" s="8" t="n">
@@ -11219,7 +11227,7 @@
       </c>
       <c r="C227" s="5" t="inlineStr">
         <is>
-          <t>bank transfer</t>
+          <t>debit card</t>
         </is>
       </c>
       <c r="D227" s="8" t="n">
@@ -11257,512 +11265,44 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="5" t="inlineStr">
-        <is>
-          <t>Instarem</t>
-        </is>
-      </c>
-      <c r="B228" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C228" s="5" t="inlineStr">
-        <is>
-          <t>debit card</t>
-        </is>
-      </c>
-      <c r="D228" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="E228" s="9" t="n">
-        <v>108.885</v>
-      </c>
-      <c r="F228" s="9" t="n"/>
-      <c r="G228" s="21" t="inlineStr">
-        <is>
-          <t>11:05</t>
-        </is>
-      </c>
-      <c r="H228" s="12" t="n">
-        <v>10875.21</v>
-      </c>
-      <c r="I228" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J228" s="9" t="n">
-        <v>108.1316</v>
-      </c>
-      <c r="K228" s="10" t="n">
-        <v>108.7521</v>
-      </c>
-      <c r="L228" s="15">
-        <f>IF(OR(E228="",J228=""),"",(E228-J228)/E228)</f>
-        <v/>
-      </c>
-      <c r="M228" s="15" t="n"/>
-      <c r="N228" s="10" t="n"/>
-      <c r="O228" s="16" t="inlineStr">
-        <is>
-          <t>First-transfer rate 108.7521 shown; regular rate 108.1316 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L228" s="22" t="n"/>
+      <c r="M228" s="22" t="n"/>
     </row>
     <row r="229">
-      <c r="A229" s="5" t="inlineStr">
-        <is>
-          <t>Instarem</t>
-        </is>
-      </c>
-      <c r="B229" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C229" s="5" t="inlineStr">
-        <is>
-          <t>debit card</t>
-        </is>
-      </c>
-      <c r="D229" s="8" t="n">
-        <v>500</v>
-      </c>
-      <c r="E229" s="9" t="n">
-        <v>108.885</v>
-      </c>
-      <c r="F229" s="9" t="n"/>
-      <c r="G229" s="21" t="inlineStr">
-        <is>
-          <t>11:05</t>
-        </is>
-      </c>
-      <c r="H229" s="12" t="n">
-        <v>54376.05</v>
-      </c>
-      <c r="I229" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J229" s="9" t="n">
-        <v>108.1752</v>
-      </c>
-      <c r="K229" s="10" t="n">
-        <v>108.7521</v>
-      </c>
-      <c r="L229" s="15">
-        <f>IF(OR(E229="",J229=""),"",(E229-J229)/E229)</f>
-        <v/>
-      </c>
-      <c r="M229" s="15" t="n"/>
-      <c r="N229" s="10" t="n"/>
-      <c r="O229" s="16" t="inlineStr">
-        <is>
-          <t>First-transfer rate 108.7521 shown; regular rate 108.1752 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L229" s="22" t="n"/>
+      <c r="M229" s="22" t="n"/>
     </row>
     <row r="230">
-      <c r="A230" s="5" t="inlineStr">
-        <is>
-          <t>Instarem</t>
-        </is>
-      </c>
-      <c r="B230" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C230" s="5" t="inlineStr">
-        <is>
-          <t>debit card</t>
-        </is>
-      </c>
-      <c r="D230" s="8" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E230" s="9" t="n">
-        <v>108.885</v>
-      </c>
-      <c r="F230" s="9" t="n"/>
-      <c r="G230" s="21" t="inlineStr">
-        <is>
-          <t>11:05</t>
-        </is>
-      </c>
-      <c r="H230" s="12" t="n">
-        <v>108752.1</v>
-      </c>
-      <c r="I230" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J230" s="9" t="n">
-        <v>108.2078</v>
-      </c>
-      <c r="K230" s="10" t="n">
-        <v>108.7521</v>
-      </c>
-      <c r="L230" s="15">
-        <f>IF(OR(E230="",J230=""),"",(E230-J230)/E230)</f>
-        <v/>
-      </c>
-      <c r="M230" s="15" t="n"/>
-      <c r="N230" s="10" t="n"/>
-      <c r="O230" s="16" t="inlineStr">
-        <is>
-          <t>First-transfer rate 108.7521 shown; regular rate 108.2078 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L230" s="22" t="n"/>
+      <c r="M230" s="22" t="n"/>
     </row>
     <row r="231">
-      <c r="A231" s="5" t="inlineStr">
-        <is>
-          <t>Instarem</t>
-        </is>
-      </c>
-      <c r="B231" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C231" s="5" t="inlineStr">
-        <is>
-          <t>debit card</t>
-        </is>
-      </c>
-      <c r="D231" s="8" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E231" s="9" t="n">
-        <v>108.885</v>
-      </c>
-      <c r="F231" s="9" t="n"/>
-      <c r="G231" s="21" t="inlineStr">
-        <is>
-          <t>11:05</t>
-        </is>
-      </c>
-      <c r="H231" s="12" t="n">
-        <v>217504.2</v>
-      </c>
-      <c r="I231" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J231" s="9" t="n">
-        <v>108.2078</v>
-      </c>
-      <c r="K231" s="10" t="n">
-        <v>108.7521</v>
-      </c>
-      <c r="L231" s="15">
-        <f>IF(OR(E231="",J231=""),"",(E231-J231)/E231)</f>
-        <v/>
-      </c>
-      <c r="M231" s="15" t="n"/>
-      <c r="N231" s="10" t="n"/>
-      <c r="O231" s="16" t="inlineStr">
-        <is>
-          <t>First-transfer rate 108.7521 shown; regular rate 108.2078 (fee 0.00) | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L231" s="22" t="n"/>
+      <c r="M231" s="22" t="n"/>
     </row>
     <row r="232">
-      <c r="A232" s="5" t="inlineStr">
-        <is>
-          <t>Instarem</t>
-        </is>
-      </c>
-      <c r="B232" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C232" s="5" t="inlineStr">
-        <is>
-          <t>debit card</t>
-        </is>
-      </c>
-      <c r="D232" s="8" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E232" s="9" t="n">
-        <v>108.885</v>
-      </c>
-      <c r="F232" s="9" t="n"/>
-      <c r="G232" s="21" t="inlineStr">
-        <is>
-          <t>11:05</t>
-        </is>
-      </c>
-      <c r="H232" s="12" t="n">
-        <v>541311.5</v>
-      </c>
-      <c r="I232" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J232" s="9" t="n">
-        <v>108.3167</v>
-      </c>
-      <c r="K232" s="10" t="n"/>
-      <c r="L232" s="15">
-        <f>IF(OR(E232="",J232=""),"",(E232-J232)/E232)</f>
-        <v/>
-      </c>
-      <c r="M232" s="15" t="n"/>
-      <c r="N232" s="10" t="n"/>
-      <c r="O232" s="16" t="inlineStr">
-        <is>
-          <t>Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L232" s="22" t="n"/>
+      <c r="M232" s="22" t="n"/>
     </row>
     <row r="233">
-      <c r="A233" s="5" t="inlineStr">
-        <is>
-          <t>Skrill</t>
-        </is>
-      </c>
-      <c r="B233" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C233" s="5" t="inlineStr">
-        <is>
-          <t>bank transfer</t>
-        </is>
-      </c>
-      <c r="D233" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="E233" s="9" t="n">
-        <v>108.893</v>
-      </c>
-      <c r="F233" s="9" t="n"/>
-      <c r="G233" s="21" t="inlineStr">
-        <is>
-          <t>11:06</t>
-        </is>
-      </c>
-      <c r="H233" s="12" t="n">
-        <v>10821.77</v>
-      </c>
-      <c r="I233" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J233" s="9" t="n">
-        <v>108.2177</v>
-      </c>
-      <c r="K233" s="10" t="n"/>
-      <c r="L233" s="15">
-        <f>IF(OR(E233="",J233=""),"",(E233-J233)/E233)</f>
-        <v/>
-      </c>
-      <c r="M233" s="15" t="n"/>
-      <c r="N233" s="10" t="n"/>
-      <c r="O233" s="16" t="inlineStr">
-        <is>
-          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L233" s="22" t="n"/>
+      <c r="M233" s="22" t="n"/>
     </row>
     <row r="234">
-      <c r="A234" s="5" t="inlineStr">
-        <is>
-          <t>Skrill</t>
-        </is>
-      </c>
-      <c r="B234" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C234" s="5" t="inlineStr">
-        <is>
-          <t>bank transfer</t>
-        </is>
-      </c>
-      <c r="D234" s="8" t="n">
-        <v>500</v>
-      </c>
-      <c r="E234" s="9" t="n">
-        <v>108.893</v>
-      </c>
-      <c r="F234" s="9" t="n"/>
-      <c r="G234" s="21" t="inlineStr">
-        <is>
-          <t>11:06</t>
-        </is>
-      </c>
-      <c r="H234" s="12" t="n">
-        <v>54108.87</v>
-      </c>
-      <c r="I234" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J234" s="9" t="n">
-        <v>108.2177</v>
-      </c>
-      <c r="K234" s="10" t="n"/>
-      <c r="L234" s="15">
-        <f>IF(OR(E234="",J234=""),"",(E234-J234)/E234)</f>
-        <v/>
-      </c>
-      <c r="M234" s="15" t="n"/>
-      <c r="N234" s="10" t="n"/>
-      <c r="O234" s="16" t="inlineStr">
-        <is>
-          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L234" s="22" t="n"/>
+      <c r="M234" s="22" t="n"/>
     </row>
     <row r="235">
-      <c r="A235" s="5" t="inlineStr">
-        <is>
-          <t>Skrill</t>
-        </is>
-      </c>
-      <c r="B235" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C235" s="5" t="inlineStr">
-        <is>
-          <t>bank transfer</t>
-        </is>
-      </c>
-      <c r="D235" s="8" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E235" s="9" t="n">
-        <v>108.893</v>
-      </c>
-      <c r="F235" s="9" t="n"/>
-      <c r="G235" s="21" t="inlineStr">
-        <is>
-          <t>11:06</t>
-        </is>
-      </c>
-      <c r="H235" s="12" t="n">
-        <v>108217.74</v>
-      </c>
-      <c r="I235" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J235" s="9" t="n">
-        <v>108.2177</v>
-      </c>
-      <c r="K235" s="10" t="n"/>
-      <c r="L235" s="15">
-        <f>IF(OR(E235="",J235=""),"",(E235-J235)/E235)</f>
-        <v/>
-      </c>
-      <c r="M235" s="15" t="n"/>
-      <c r="N235" s="10" t="n"/>
-      <c r="O235" s="16" t="inlineStr">
-        <is>
-          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L235" s="22" t="n"/>
+      <c r="M235" s="22" t="n"/>
     </row>
     <row r="236">
-      <c r="A236" s="5" t="inlineStr">
-        <is>
-          <t>Skrill</t>
-        </is>
-      </c>
-      <c r="B236" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C236" s="5" t="inlineStr">
-        <is>
-          <t>bank transfer</t>
-        </is>
-      </c>
-      <c r="D236" s="8" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E236" s="9" t="n">
-        <v>108.893</v>
-      </c>
-      <c r="F236" s="9" t="n"/>
-      <c r="G236" s="21" t="inlineStr">
-        <is>
-          <t>11:06</t>
-        </is>
-      </c>
-      <c r="H236" s="12" t="n">
-        <v>216435.47</v>
-      </c>
-      <c r="I236" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J236" s="9" t="n">
-        <v>108.2177</v>
-      </c>
-      <c r="K236" s="10" t="n"/>
-      <c r="L236" s="15">
-        <f>IF(OR(E236="",J236=""),"",(E236-J236)/E236)</f>
-        <v/>
-      </c>
-      <c r="M236" s="15" t="n"/>
-      <c r="N236" s="10" t="n"/>
-      <c r="O236" s="16" t="inlineStr">
-        <is>
-          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L236" s="22" t="n"/>
+      <c r="M236" s="22" t="n"/>
     </row>
     <row r="237">
-      <c r="A237" s="5" t="inlineStr">
-        <is>
-          <t>Skrill</t>
-        </is>
-      </c>
-      <c r="B237" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C237" s="5" t="inlineStr">
-        <is>
-          <t>bank transfer</t>
-        </is>
-      </c>
-      <c r="D237" s="8" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E237" s="9" t="n">
-        <v>108.893</v>
-      </c>
-      <c r="F237" s="9" t="n"/>
-      <c r="G237" s="21" t="inlineStr">
-        <is>
-          <t>11:06</t>
-        </is>
-      </c>
-      <c r="H237" s="12" t="n">
-        <v>541088.6800000001</v>
-      </c>
-      <c r="I237" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J237" s="9" t="n">
-        <v>108.2177</v>
-      </c>
-      <c r="K237" s="10" t="n"/>
-      <c r="L237" s="15">
-        <f>IF(OR(E237="",J237=""),"",(E237-J237)/E237)</f>
-        <v/>
-      </c>
-      <c r="M237" s="15" t="n"/>
-      <c r="N237" s="10" t="n"/>
-      <c r="O237" s="16" t="inlineStr">
-        <is>
-          <t>Estimate from Wise comparison data (collected 2026-09-30, DE), not a live quote | Auto-scraped; mid rate = Wise live mid</t>
-        </is>
-      </c>
+      <c r="L237" s="22" t="n"/>
+      <c r="M237" s="22" t="n"/>
     </row>
     <row r="238">
       <c r="L238" s="22" t="n"/>
@@ -14711,46 +14251,6 @@
     <row r="974">
       <c r="L974" s="22" t="n"/>
       <c r="M974" s="22" t="n"/>
-    </row>
-    <row r="975">
-      <c r="L975" s="22" t="n"/>
-      <c r="M975" s="22" t="n"/>
-    </row>
-    <row r="976">
-      <c r="L976" s="22" t="n"/>
-      <c r="M976" s="22" t="n"/>
-    </row>
-    <row r="977">
-      <c r="L977" s="22" t="n"/>
-      <c r="M977" s="22" t="n"/>
-    </row>
-    <row r="978">
-      <c r="L978" s="22" t="n"/>
-      <c r="M978" s="22" t="n"/>
-    </row>
-    <row r="979">
-      <c r="L979" s="22" t="n"/>
-      <c r="M979" s="22" t="n"/>
-    </row>
-    <row r="980">
-      <c r="L980" s="22" t="n"/>
-      <c r="M980" s="22" t="n"/>
-    </row>
-    <row r="981">
-      <c r="L981" s="22" t="n"/>
-      <c r="M981" s="22" t="n"/>
-    </row>
-    <row r="982">
-      <c r="L982" s="22" t="n"/>
-      <c r="M982" s="22" t="n"/>
-    </row>
-    <row r="983">
-      <c r="L983" s="22" t="n"/>
-      <c r="M983" s="22" t="n"/>
-    </row>
-    <row r="984">
-      <c r="L984" s="22" t="n"/>
-      <c r="M984" s="22" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>